<commit_message>
puta weekend dayoff trabaho pa rin
</commit_message>
<xml_diff>
--- a/Documents/devfiles/excel/DBdesignVer2.xlsx
+++ b/Documents/devfiles/excel/DBdesignVer2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\devfiles\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Gitlab\joboffer\Documents\devfiles\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F85D16D-AD4D-4D1B-9C2F-0146C6C881A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44AF28B3-5EB0-421D-851D-F3ACCC99BF35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="23040" windowHeight="12120" activeTab="6" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
   </bookViews>
   <sheets>
     <sheet name="ReferenceTable" sheetId="12" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Letter" sheetId="15" r:id="rId4"/>
     <sheet name="Status" sheetId="16" r:id="rId5"/>
     <sheet name="StatusName" sheetId="17" r:id="rId6"/>
-    <sheet name="Draft" sheetId="18" r:id="rId7"/>
+    <sheet name="Draft" sheetId="19" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="109">
   <si>
     <t>Name</t>
   </si>
@@ -359,76 +359,19 @@
     <t>EmailTemplate</t>
   </si>
   <si>
-    <t>Message</t>
-  </si>
-  <si>
-    <t>TemplateId</t>
-  </si>
-  <si>
     <t>OtherRecipient</t>
   </si>
   <si>
-    <t>by</t>
-  </si>
-  <si>
-    <t>[ Roles Dropdown ]</t>
-  </si>
-  <si>
-    <t>[ Actions  Dropdown ]</t>
-  </si>
-  <si>
-    <t>Template Name</t>
-  </si>
-  <si>
-    <t>Recipients</t>
-  </si>
-  <si>
-    <t>TA Partner</t>
-  </si>
-  <si>
-    <t>TA Lead</t>
-  </si>
-  <si>
-    <t>PE Head</t>
-  </si>
-  <si>
-    <t>HROD Head Approver</t>
-  </si>
-  <si>
-    <t>Division Head Approver L1</t>
-  </si>
-  <si>
-    <t>Division Head Approver L2</t>
-  </si>
-  <si>
-    <t>President</t>
-  </si>
-  <si>
-    <t>Business Admin</t>
-  </si>
-  <si>
-    <t>Onboarding Partner</t>
-  </si>
-  <si>
-    <t>System Administrator</t>
-  </si>
-  <si>
-    <t>Others:</t>
-  </si>
-  <si>
     <t>EmailSubect</t>
   </si>
   <si>
     <t>EmailMessage</t>
   </si>
   <si>
-    <t>EmailAddress</t>
-  </si>
-  <si>
     <t>EmailTemplateRoles</t>
   </si>
   <si>
-    <t>EmailTemplateRecipients</t>
+    <t>EmailTemplateId</t>
   </si>
 </sst>
 </file>
@@ -473,7 +416,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -481,106 +424,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -595,23 +443,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -947,16 +778,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD3E0DE8-4720-4CDB-8DB3-CDF187788EC3}">
   <dimension ref="B2:J21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.1796875" customWidth="1"/>
-    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.21875" customWidth="1"/>
+    <col min="6" max="6" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
@@ -973,7 +804,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -990,7 +821,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>4</v>
       </c>
@@ -1007,12 +838,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>25</v>
       </c>
@@ -1023,7 +854,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>5</v>
       </c>
@@ -1037,7 +868,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>26</v>
       </c>
@@ -1048,7 +879,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>27</v>
       </c>
@@ -1062,7 +893,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
         <v>5</v>
       </c>
@@ -1073,7 +904,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D11" t="s">
         <v>19</v>
       </c>
@@ -1084,7 +915,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
         <v>10</v>
       </c>
@@ -1092,37 +923,37 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H15" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H16" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H17" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H18" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="8:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H20" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H21" s="2" t="s">
         <v>7</v>
       </c>
@@ -1135,13 +966,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5710F30C-E88B-4A3C-8A63-0D8128BE2FFF}">
   <dimension ref="B2:D11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>37</v>
       </c>
@@ -1149,7 +980,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>38</v>
       </c>
@@ -1157,7 +988,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>1</v>
       </c>
@@ -1165,32 +996,32 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D5" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>42</v>
       </c>
@@ -1203,15 +1034,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE7AE70E-E5CC-4406-BB70-6FBBBFBDDCCE}">
   <dimension ref="B2:H26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.90625" customWidth="1"/>
-    <col min="6" max="6" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.88671875" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>29</v>
       </c>
@@ -1225,7 +1056,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>5</v>
       </c>
@@ -1239,7 +1070,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -1250,7 +1081,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>45</v>
       </c>
@@ -1258,12 +1089,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="D6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>30</v>
       </c>
@@ -1271,7 +1102,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>31</v>
       </c>
@@ -1279,7 +1110,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>24</v>
       </c>
@@ -1287,7 +1118,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>32</v>
       </c>
@@ -1295,7 +1126,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>33</v>
       </c>
@@ -1303,7 +1134,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>34</v>
       </c>
@@ -1311,7 +1142,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>35</v>
       </c>
@@ -1319,12 +1150,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
       <c r="D14" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>36</v>
       </c>
@@ -1332,7 +1163,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>11</v>
       </c>
@@ -1340,12 +1171,12 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>13</v>
       </c>
@@ -1353,12 +1184,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D19" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>43</v>
       </c>
@@ -1366,7 +1197,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>7</v>
       </c>
@@ -1374,27 +1205,27 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D22" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D24" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D25" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D26" t="s">
         <v>82</v>
       </c>
@@ -1407,16 +1238,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C2552A1-D2D6-4D6E-936E-AAD262657723}">
   <dimension ref="B2:H26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.1796875" customWidth="1"/>
-    <col min="6" max="6" width="19.453125" customWidth="1"/>
-    <col min="8" max="8" width="22.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.21875" customWidth="1"/>
+    <col min="6" max="6" width="19.44140625" customWidth="1"/>
+    <col min="8" max="8" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>36</v>
       </c>
@@ -1427,10 +1258,10 @@
         <v>103</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>11</v>
       </c>
@@ -1438,13 +1269,13 @@
         <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="H3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>44</v>
       </c>
@@ -1452,13 +1283,13 @@
         <v>60</v>
       </c>
       <c r="F4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4" t="s">
         <v>42</v>
       </c>
-      <c r="H4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>13</v>
       </c>
@@ -1466,123 +1297,108 @@
         <v>13</v>
       </c>
       <c r="F5" t="s">
-        <v>74</v>
-      </c>
-      <c r="H5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
-        <v>106</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F8" t="s">
-        <v>6</v>
-      </c>
-      <c r="H8" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>47</v>
       </c>
-      <c r="H9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>45</v>
       </c>
@@ -1595,16 +1411,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BADF9B9-38B5-461D-B650-FB9B2CB7966D}">
   <dimension ref="B2:J10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>67</v>
       </c>
@@ -1621,7 +1437,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>68</v>
       </c>
@@ -1638,7 +1454,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D4" t="s">
         <v>73</v>
       </c>
@@ -1652,7 +1468,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>62</v>
       </c>
@@ -1669,7 +1485,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>63</v>
       </c>
@@ -1683,7 +1499,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
         <v>98</v>
       </c>
@@ -1691,12 +1507,12 @@
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>69</v>
       </c>
@@ -1709,14 +1525,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ABED4AD-1AED-4632-9454-063816F78CB2}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.36328125" customWidth="1"/>
-    <col min="3" max="3" width="72.90625" customWidth="1"/>
+    <col min="1" max="1" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.33203125" customWidth="1"/>
+    <col min="3" max="3" width="72.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>83</v>
       </c>
@@ -1727,7 +1543,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="B2" s="4" t="s">
         <v>86</v>
@@ -1736,7 +1552,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
         <v>88</v>
@@ -1745,7 +1561,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
         <v>97</v>
@@ -1754,7 +1570,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
         <v>90</v>
@@ -1763,7 +1579,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="4" t="s">
         <v>92</v>
@@ -1772,7 +1588,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="4" t="s">
         <v>94</v>
@@ -1781,7 +1597,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="4" t="s">
         <v>96</v>
@@ -1794,182 +1610,10 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{962C5333-1C8B-4B37-8B21-2BB34F0D737A}">
-  <dimension ref="A1:M21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" customWidth="1"/>
-    <col min="3" max="3" width="21.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.26953125" customWidth="1"/>
-    <col min="5" max="5" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.90625" customWidth="1"/>
-    <col min="11" max="11" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.1796875" customWidth="1"/>
-    <col min="13" max="13" width="12.7265625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" s="7"/>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="7"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C4" s="13"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="14"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C5" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="14"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C6" s="15"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="17"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C9" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="D9" s="19"/>
-      <c r="E9" s="20" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C10" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="14"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C11" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="14"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C12" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="14"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C13" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D13" s="7"/>
-      <c r="E13" s="14"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C14" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="14"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C15" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="D15" s="7"/>
-      <c r="E15" s="14"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="C16" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="14"/>
-    </row>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.35">
-      <c r="C17" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="D17" s="7"/>
-      <c r="E17" s="14"/>
-    </row>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.35">
-      <c r="C18" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="D18" s="7"/>
-      <c r="E18" s="14"/>
-    </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.35">
-      <c r="C19" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="D19" s="7"/>
-      <c r="E19" s="14"/>
-    </row>
-    <row r="20" spans="3:5" x14ac:dyDescent="0.35">
-      <c r="C20" s="13"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="14"/>
-    </row>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.35">
-      <c r="C21" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="D21" s="16"/>
-      <c r="E21" s="17"/>
-    </row>
-  </sheetData>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B7B37E1-E9C8-4011-B172-9D118CCEF591}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>